<commit_message>
P5 step 2: linked card payments at the till (DL-218..220)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P5.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P5.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -875,9 +875,324 @@
       <c r="H9" s="3" t="inlineStr"/>
       <c r="I9" s="3" t="inlineStr"/>
     </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Linked card</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Till with a terminal</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Sell an item → Pay → Card → Send to the terminal</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>The terminal shows the amount; the till says Waiting for the card</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr"/>
+      <c r="H10" s="3" t="inlineStr"/>
+      <c r="I10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>C11</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Linked card</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Pay with the sandbox card (or tap a card)</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Within seconds the till adds Card ****1111 · terminal; the sale completes; the receipt shows the card</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr"/>
+      <c r="I11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>C12</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Linked card</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Card → Send → Cancel on the till</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>The terminal goes back to idle; the till says Cancelled; Try again works</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
+      <c r="H12" s="3" t="inlineStr"/>
+      <c r="I12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Linked card</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Card → Send; cancel on the terminal</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>The till says the customer cancelled; Key it in instead opens the old dialog</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr"/>
+      <c r="I13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>C14</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Linked card</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Split: Card $5.00 on the terminal, the rest cash</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Both payments on the receipt</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr"/>
+      <c r="H14" s="3" t="inlineStr"/>
+      <c r="I14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>C15</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Linked card</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Card → Send, pay on the terminal, then reload the page before the sale completes; press Pay</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>The card payment is back in the payments (a note says so); the sale completes without charging again</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr"/>
+      <c r="H15" s="3" t="inlineStr"/>
+      <c r="I15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>C16</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Linked card</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Switch the router's internet off; Card</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>The till shows Could not reach the terminal → Key it in instead works</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr"/>
+      <c r="H16" s="3" t="inlineStr"/>
+      <c r="I16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Linked card</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Training mode on; Card</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>The old dialog (training never charges a card)</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr"/>
+      <c r="H17" s="3" t="inlineStr"/>
+      <c r="I17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>C18</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Linked card</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Till without a terminal</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>The old dialog: key the amount in</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr"/>
+      <c r="H18" s="3" t="inlineStr"/>
+      <c r="I18" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I9"/>
-  <conditionalFormatting sqref="F2:F9">
+  <autoFilter ref="A1:I18"/>
+  <conditionalFormatting sqref="F2:F18">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -892,7 +1207,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -906,7 +1221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -977,29 +1292,56 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Linked card</t>
+        </is>
+      </c>
+      <c r="B3">
+        <f>COUNTIF(Tests!B:B,A3)</f>
+        <v/>
+      </c>
+      <c r="C3">
+        <f>COUNTIFS(Tests!B:B,A3,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D3">
+        <f>COUNTIFS(Tests!B:B,A3,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E3">
+        <f>COUNTIFS(Tests!B:B,A3,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F3">
+        <f>COUNTIFS(Tests!B:B,A3,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B3" s="5">
-        <f>SUM(B2:B2)</f>
-        <v/>
-      </c>
-      <c r="C3" s="5">
-        <f>SUM(C2:C2)</f>
-        <v/>
-      </c>
-      <c r="D3" s="5">
-        <f>SUM(D2:D2)</f>
-        <v/>
-      </c>
-      <c r="E3" s="5">
-        <f>SUM(E2:E2)</f>
-        <v/>
-      </c>
-      <c r="F3" s="5">
-        <f>SUM(F2:F2)</f>
+      <c r="B4" s="5">
+        <f>SUM(B2:B3)</f>
+        <v/>
+      </c>
+      <c r="C4" s="5">
+        <f>SUM(C2:C3)</f>
+        <v/>
+      </c>
+      <c r="D4" s="5">
+        <f>SUM(D2:D3)</f>
+        <v/>
+      </c>
+      <c r="E4" s="5">
+        <f>SUM(E2:E3)</f>
+        <v/>
+      </c>
+      <c r="F4" s="5">
+        <f>SUM(F2:F3)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
P5 step 3: card refunds through the processor, fees and payouts (DL-221..223)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P5.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P5.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1190,9 +1190,219 @@
       <c r="H18" s="3" t="inlineStr"/>
       <c r="I18" s="3" t="inlineStr"/>
     </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>C20</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Linked refund</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Sell 2 items paid on the terminal (Visa); Sell → Return → 1 item → Back to the card</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Refunded without the card; the return slip shows Card ****… · back to the card; Square shows the refund</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr"/>
+      <c r="H19" s="3" t="inlineStr"/>
+      <c r="I19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>C21</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Linked refund</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Till + terminal</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>A sale paid by debit (Interac) on the terminal; return it → Back to the card</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>The till says: Customer, tap or insert the card; after the tap the return completes</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr"/>
+      <c r="H20" s="3" t="inlineStr"/>
+      <c r="I20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>C22</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Linked refund</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Till</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Start a return Back to the card, then reload the page and do the same return again</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>The refund already made comes back (no second refund in Square)</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr"/>
+      <c r="H21" s="3" t="inlineStr"/>
+      <c r="I21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>C23</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Linked void</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Till (manager)</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Void the last sale that was paid on the terminal</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Asks first; the money goes back to the card; then the sale is voided</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr"/>
+      <c r="H22" s="3" t="inlineStr"/>
+      <c r="I22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>C24</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Unused payment</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Till + laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Card → Send, pay on the terminal, then Clear sale (OK); after 15 minutes open Sales</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Card payments taken on the terminal with no sale: the payment → Refund to the card</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr"/>
+      <c r="H23" s="3" t="inlineStr"/>
+      <c r="I23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>C25</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Fees</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (accountant)</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Fees and statements → Card fees → Get fees and payouts now</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>From the linked card processor: the fees; payouts listed with their dates</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr"/>
+      <c r="H24" s="3" t="inlineStr"/>
+      <c r="I24" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I18"/>
-  <conditionalFormatting sqref="F2:F18">
+  <autoFilter ref="A1:I24"/>
+  <conditionalFormatting sqref="F2:F24">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -1207,7 +1417,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1221,7 +1431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1319,29 +1529,137 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Linked refund</t>
+        </is>
+      </c>
+      <c r="B4">
+        <f>COUNTIF(Tests!B:B,A4)</f>
+        <v/>
+      </c>
+      <c r="C4">
+        <f>COUNTIFS(Tests!B:B,A4,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D4">
+        <f>COUNTIFS(Tests!B:B,A4,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E4">
+        <f>COUNTIFS(Tests!B:B,A4,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F4">
+        <f>COUNTIFS(Tests!B:B,A4,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Linked void</t>
+        </is>
+      </c>
+      <c r="B5">
+        <f>COUNTIF(Tests!B:B,A5)</f>
+        <v/>
+      </c>
+      <c r="C5">
+        <f>COUNTIFS(Tests!B:B,A5,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D5">
+        <f>COUNTIFS(Tests!B:B,A5,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E5">
+        <f>COUNTIFS(Tests!B:B,A5,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F5">
+        <f>COUNTIFS(Tests!B:B,A5,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Unused payment</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>COUNTIF(Tests!B:B,A6)</f>
+        <v/>
+      </c>
+      <c r="C6">
+        <f>COUNTIFS(Tests!B:B,A6,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D6">
+        <f>COUNTIFS(Tests!B:B,A6,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E6">
+        <f>COUNTIFS(Tests!B:B,A6,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F6">
+        <f>COUNTIFS(Tests!B:B,A6,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Fees</t>
+        </is>
+      </c>
+      <c r="B7">
+        <f>COUNTIF(Tests!B:B,A7)</f>
+        <v/>
+      </c>
+      <c r="C7">
+        <f>COUNTIFS(Tests!B:B,A7,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D7">
+        <f>COUNTIFS(Tests!B:B,A7,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E7">
+        <f>COUNTIFS(Tests!B:B,A7,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F7">
+        <f>COUNTIFS(Tests!B:B,A7,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B4" s="5">
-        <f>SUM(B2:B3)</f>
-        <v/>
-      </c>
-      <c r="C4" s="5">
-        <f>SUM(C2:C3)</f>
-        <v/>
-      </c>
-      <c r="D4" s="5">
-        <f>SUM(D2:D3)</f>
-        <v/>
-      </c>
-      <c r="E4" s="5">
-        <f>SUM(E2:E3)</f>
-        <v/>
-      </c>
-      <c r="F4" s="5">
-        <f>SUM(F2:F3)</f>
+      <c r="B8" s="5">
+        <f>SUM(B2:B7)</f>
+        <v/>
+      </c>
+      <c r="C8" s="5">
+        <f>SUM(C2:C7)</f>
+        <v/>
+      </c>
+      <c r="D8" s="5">
+        <f>SUM(D2:D7)</f>
+        <v/>
+      </c>
+      <c r="E8" s="5">
+        <f>SUM(E2:E7)</f>
+        <v/>
+      </c>
+      <c r="F8" s="5">
+        <f>SUM(F2:F7)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
P5 step 4: cloud drive by device code, off-site backup copy (DL-224, 225)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P5.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P5.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1400,9 +1400,219 @@
       <c r="H24" s="3" t="inlineStr"/>
       <c r="I24" s="3" t="inlineStr"/>
     </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>D01</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Cloud drive</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (owner)</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Home → Cloud drive → Google Drive → Enter the client ID and secret → Save</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>App registration: client ID 1234…; the secret is not shown</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr"/>
+      <c r="H25" s="3" t="inlineStr"/>
+      <c r="I25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>D02</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Cloud drive</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (owner) + phone</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Connect Google Drive; on the phone open google.com/device, type the code, allow</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Within seconds the laptop says Google Drive is connected, with the owner's email</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr"/>
+      <c r="H26" s="3" t="inlineStr"/>
+      <c r="I26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>D03</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Cloud drive</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (owner)</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Backups → Back up now; then Cloud drive → Upload now</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Last backup copied: chedam-…db.gz.age; in Google Drive a 'Chedam' folder has the backup and its .keys/.ca/.sha256</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr"/>
+      <c r="H27" s="3" t="inlineStr"/>
+      <c r="I27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>D04</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Cloud drive</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Google account</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Remove Chedam's access in the Google account's security page; next upload</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Cloud drive says: connect the cloud drive again; the backup waits in the outbox</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr"/>
+      <c r="H28" s="3" t="inlineStr"/>
+      <c r="I28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>D05</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Cloud drive</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (owner)</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Disconnect; connect OneDrive the same way (microsoft.com/devicelogin)</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Connected; the next backup is in OneDrive → Apps → Chedam</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr"/>
+      <c r="H29" s="3" t="inlineStr"/>
+      <c r="I29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>D06</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Cloud drive</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Look for Cloud drive on Home</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>No tile (owner only)</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr"/>
+      <c r="H30" s="3" t="inlineStr"/>
+      <c r="I30" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I24"/>
-  <conditionalFormatting sqref="F2:F24">
+  <autoFilter ref="A1:I30"/>
+  <conditionalFormatting sqref="F2:F30">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -1417,7 +1627,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1431,7 +1641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1637,29 +1847,56 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Cloud drive</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>COUNTIF(Tests!B:B,A8)</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>COUNTIFS(Tests!B:B,A8,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>COUNTIFS(Tests!B:B,A8,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>COUNTIFS(Tests!B:B,A8,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>COUNTIFS(Tests!B:B,A8,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B8" s="5">
-        <f>SUM(B2:B7)</f>
-        <v/>
-      </c>
-      <c r="C8" s="5">
-        <f>SUM(C2:C7)</f>
-        <v/>
-      </c>
-      <c r="D8" s="5">
-        <f>SUM(D2:D7)</f>
-        <v/>
-      </c>
-      <c r="E8" s="5">
-        <f>SUM(E2:E7)</f>
-        <v/>
-      </c>
-      <c r="F8" s="5">
-        <f>SUM(F2:F7)</f>
+      <c r="B9" s="5">
+        <f>SUM(B2:B8)</f>
+        <v/>
+      </c>
+      <c r="C9" s="5">
+        <f>SUM(C2:C8)</f>
+        <v/>
+      </c>
+      <c r="D9" s="5">
+        <f>SUM(D2:D8)</f>
+        <v/>
+      </c>
+      <c r="E9" s="5">
+        <f>SUM(E2:E8)</f>
+        <v/>
+      </c>
+      <c r="F9" s="5">
+        <f>SUM(F2:F8)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
P5 step 5: owner's remote view, encrypted summary on the cloud drive (DL-226..228)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P5.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P5.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1610,9 +1610,184 @@
       <c r="H30" s="3" t="inlineStr"/>
       <c r="I30" s="3" t="inlineStr"/>
     </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Remote view</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (owner)</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Cloud drive → Send the summary now</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Last: now; in the cloud drive a file chedam-summary.enc (its content is unreadable)</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr"/>
+      <c r="H31" s="3" t="inlineStr"/>
+      <c r="I31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>D11</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Remote view</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>iPhone (owner, at the store)</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Home → Cloud drive → Enrol this device → Open the remote view</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Today's sales, tills open, who is clocked in, attention, stock, last backup; Last updated with the time</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr"/>
+      <c r="H32" s="3" t="inlineStr"/>
+      <c r="I32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Remote view</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>iPhone (owner, on mobile data, away)</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Turn Wi-Fi off; open Chedam from the home screen</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>The bar says the hub can't be reached; the link Away from the store? See the latest summary opens it</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr"/>
+      <c r="H33" s="3" t="inlineStr"/>
+      <c r="I33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Remote view</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>iPhone (owner, away)</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Sell something at the store; 15 minutes later press Refresh</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>The sale is in today's total; the time is newer</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr"/>
+      <c r="H34" s="3" t="inlineStr"/>
+      <c r="I34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>D14</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Remote view</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (owner)</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Forget enrolled devices; on the iPhone (away) press Refresh after the next summary</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>The iPhone says to enrol this device again</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr"/>
+      <c r="H35" s="3" t="inlineStr"/>
+      <c r="I35" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I30"/>
-  <conditionalFormatting sqref="F2:F30">
+  <autoFilter ref="A1:I35"/>
+  <conditionalFormatting sqref="F2:F35">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -1627,7 +1802,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1641,7 +1816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1874,29 +2049,56 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Remote view</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>COUNTIF(Tests!B:B,A9)</f>
+        <v/>
+      </c>
+      <c r="C9">
+        <f>COUNTIFS(Tests!B:B,A9,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D9">
+        <f>COUNTIFS(Tests!B:B,A9,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>COUNTIFS(Tests!B:B,A9,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F9">
+        <f>COUNTIFS(Tests!B:B,A9,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B9" s="5">
-        <f>SUM(B2:B8)</f>
-        <v/>
-      </c>
-      <c r="C9" s="5">
-        <f>SUM(C2:C8)</f>
-        <v/>
-      </c>
-      <c r="D9" s="5">
-        <f>SUM(D2:D8)</f>
-        <v/>
-      </c>
-      <c r="E9" s="5">
-        <f>SUM(E2:E8)</f>
-        <v/>
-      </c>
-      <c r="F9" s="5">
-        <f>SUM(F2:F8)</f>
+      <c r="B10" s="5">
+        <f>SUM(B2:B9)</f>
+        <v/>
+      </c>
+      <c r="C10" s="5">
+        <f>SUM(C2:C9)</f>
+        <v/>
+      </c>
+      <c r="D10" s="5">
+        <f>SUM(D2:D9)</f>
+        <v/>
+      </c>
+      <c r="E10" s="5">
+        <f>SUM(E2:E9)</f>
+        <v/>
+      </c>
+      <c r="F10" s="5">
+        <f>SUM(F2:F9)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
P5 step 6: import every kind of record, mapping templates for other systems (DL-229..231)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P5.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P5.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1785,9 +1785,324 @@
       <c r="H35" s="3" t="inlineStr"/>
       <c r="I35" s="3" t="inlineStr"/>
     </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>I01</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Import products</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Import and export → Import products: a Shopify products CSV (or Square item library)</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Step 2 says the columns look like an export from Shopify; name, price, barcode, cost already mapped</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr"/>
+      <c r="H36" s="3" t="inlineStr"/>
+      <c r="I36" s="3" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>I02</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Import products</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Map an unknown sheet by hand; Save this mapping as a template 'Our sheet'; import the same layout again</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>The second time: 'your template Our sheet', mapped by itself</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr"/>
+      <c r="H37" s="3" t="inlineStr"/>
+      <c r="I37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>I03</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Import customers</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Import other records → Customers: a Square customer export, without ticking 'agreed'</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Check: every row says to confirm they agreed</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr"/>
+      <c r="H38" s="3" t="inlineStr"/>
+      <c r="I38" s="3" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>I04</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Import customers</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Tick 'agreed'; check; import</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>New members with their points; found at the till by phone</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr"/>
+      <c r="H39" s="3" t="inlineStr"/>
+      <c r="I39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>I05</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Import vendors</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Vendors and clients: a QuickBooks vendor list</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>QuickBooks recognised; vendors with terms and contact; importing again: already there</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr"/>
+      <c r="H40" s="3" t="inlineStr"/>
+      <c r="I40" s="3" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>I06</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Opening stock</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Opening stock: barcode + quantity + cost for new products</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Stock shows the quantities; Stock history: receive 'Opening stock (import)'; products that had stock are skipped</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr"/>
+      <c r="H41" s="3" t="inlineStr"/>
+      <c r="I41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>I07</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Open bills</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (accountant)</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Open bills and invoices: a QuickBooks A/P aging (Vendor, Num, Due date, Open balance)</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Bills with 'Opening balance' lines, no tax, due dates; in Buying → Bills and the aging</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr"/>
+      <c r="H42" s="3" t="inlineStr"/>
+      <c r="I42" s="3" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>I08</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Import staff</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (owner)</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Staff: name, legal name, role, start date, rate, SIN</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>People listed with their records (SIN masked); they can be paired and choose a PIN; a manager does not see Staff in the list</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr"/>
+      <c r="H43" s="3" t="inlineStr"/>
+      <c r="I43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>I09</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Export</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (owner)</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Export data: pick only 'Card processor and cloud drive'</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>The tables are there; no token or secret columns</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr"/>
+      <c r="H44" s="3" t="inlineStr"/>
+      <c r="I44" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I35"/>
-  <conditionalFormatting sqref="F2:F35">
+  <autoFilter ref="A1:I44"/>
+  <conditionalFormatting sqref="F2:F44">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -1802,7 +2117,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1816,7 +2131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2076,29 +2391,218 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Import products</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>COUNTIF(Tests!B:B,A10)</f>
+        <v/>
+      </c>
+      <c r="C10">
+        <f>COUNTIFS(Tests!B:B,A10,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D10">
+        <f>COUNTIFS(Tests!B:B,A10,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E10">
+        <f>COUNTIFS(Tests!B:B,A10,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F10">
+        <f>COUNTIFS(Tests!B:B,A10,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Import customers</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>COUNTIF(Tests!B:B,A11)</f>
+        <v/>
+      </c>
+      <c r="C11">
+        <f>COUNTIFS(Tests!B:B,A11,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D11">
+        <f>COUNTIFS(Tests!B:B,A11,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E11">
+        <f>COUNTIFS(Tests!B:B,A11,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F11">
+        <f>COUNTIFS(Tests!B:B,A11,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Import vendors</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>COUNTIF(Tests!B:B,A12)</f>
+        <v/>
+      </c>
+      <c r="C12">
+        <f>COUNTIFS(Tests!B:B,A12,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D12">
+        <f>COUNTIFS(Tests!B:B,A12,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E12">
+        <f>COUNTIFS(Tests!B:B,A12,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F12">
+        <f>COUNTIFS(Tests!B:B,A12,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Opening stock</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>COUNTIF(Tests!B:B,A13)</f>
+        <v/>
+      </c>
+      <c r="C13">
+        <f>COUNTIFS(Tests!B:B,A13,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D13">
+        <f>COUNTIFS(Tests!B:B,A13,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E13">
+        <f>COUNTIFS(Tests!B:B,A13,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F13">
+        <f>COUNTIFS(Tests!B:B,A13,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Open bills</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>COUNTIF(Tests!B:B,A14)</f>
+        <v/>
+      </c>
+      <c r="C14">
+        <f>COUNTIFS(Tests!B:B,A14,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D14">
+        <f>COUNTIFS(Tests!B:B,A14,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E14">
+        <f>COUNTIFS(Tests!B:B,A14,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F14">
+        <f>COUNTIFS(Tests!B:B,A14,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Import staff</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>COUNTIF(Tests!B:B,A15)</f>
+        <v/>
+      </c>
+      <c r="C15">
+        <f>COUNTIFS(Tests!B:B,A15,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D15">
+        <f>COUNTIFS(Tests!B:B,A15,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E15">
+        <f>COUNTIFS(Tests!B:B,A15,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F15">
+        <f>COUNTIFS(Tests!B:B,A15,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Export</t>
+        </is>
+      </c>
+      <c r="B16">
+        <f>COUNTIF(Tests!B:B,A16)</f>
+        <v/>
+      </c>
+      <c r="C16">
+        <f>COUNTIFS(Tests!B:B,A16,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D16">
+        <f>COUNTIFS(Tests!B:B,A16,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E16">
+        <f>COUNTIFS(Tests!B:B,A16,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F16">
+        <f>COUNTIFS(Tests!B:B,A16,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B10" s="5">
-        <f>SUM(B2:B9)</f>
-        <v/>
-      </c>
-      <c r="C10" s="5">
-        <f>SUM(C2:C9)</f>
-        <v/>
-      </c>
-      <c r="D10" s="5">
-        <f>SUM(D2:D9)</f>
-        <v/>
-      </c>
-      <c r="E10" s="5">
-        <f>SUM(E2:E9)</f>
-        <v/>
-      </c>
-      <c r="F10" s="5">
-        <f>SUM(F2:F9)</f>
+      <c r="B17" s="5">
+        <f>SUM(B2:B16)</f>
+        <v/>
+      </c>
+      <c r="C17" s="5">
+        <f>SUM(C2:C16)</f>
+        <v/>
+      </c>
+      <c r="D17" s="5">
+        <f>SUM(D2:D16)</f>
+        <v/>
+      </c>
+      <c r="E17" s="5">
+        <f>SUM(E2:E16)</f>
+        <v/>
+      </c>
+      <c r="F17" s="5">
+        <f>SUM(F2:F16)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
P5 step 7: reference data that suggests: datasets with the hub, Open Food Facts and Bank of Canada online, About and licences (DL-232..234)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P5.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P5.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2100,9 +2100,254 @@
       <c r="H44" s="3" t="inlineStr"/>
       <c r="I44" s="3" t="inlineStr"/>
     </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>R01</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>New product: barcode of a packaged food (e.g. a cracker box); Suggest from the barcode</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Name with the brand, French name and size from Open Food Facts, each with Use; nothing changes until Use</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr"/>
+      <c r="H45" s="3" t="inlineStr"/>
+      <c r="I45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>R02</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Same with the hub offline (router internet off)</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Not available: the hub is offline</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr"/>
+      <c r="H46" s="3" t="inlineStr"/>
+      <c r="I46" s="3" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>R03</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Product '2% Milk 4L', perishable → Shelf life → Suggest</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>Milk: 7 in the fridge … Use 7 fills 7</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr"/>
+      <c r="H47" s="3" t="inlineStr"/>
+      <c r="I47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>R04</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Imported product → HS → Find 'chocolate'</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>18 · Cocoa and chocolate (HS chapter) → Use</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr"/>
+      <c r="H48" s="3" t="inlineStr"/>
+      <c r="I48" s="3" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>R05</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Vendors and clients → Exchange rates → Add a rate: USD, last Sunday → Suggest the Bank of Canada rate</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Friday's rate with its day → Use fills the rate and the source</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr"/>
+      <c r="H49" s="3" t="inlineStr"/>
+      <c r="I49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>R06</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (owner)</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Tax → Show the sales tax rates of every province</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>13 provinces and territories (BC 5% + PST 7%, ON HST 13%, NS HST 14%); the store's own rates unchanged</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr"/>
+      <c r="H50" s="3" t="inlineStr"/>
+      <c r="I50" s="3" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>R07</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Any device</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Help → About Chedam, reference data and licences</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Version, the 4 datasets and the 2 online sources with their licences</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr"/>
+      <c r="H51" s="3" t="inlineStr"/>
+      <c r="I51" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I44"/>
-  <conditionalFormatting sqref="F2:F44">
+  <autoFilter ref="A1:I51"/>
+  <conditionalFormatting sqref="F2:F51">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -2117,7 +2362,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2131,7 +2376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2580,29 +2825,56 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>COUNTIF(Tests!B:B,A17)</f>
+        <v/>
+      </c>
+      <c r="C17">
+        <f>COUNTIFS(Tests!B:B,A17,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D17">
+        <f>COUNTIFS(Tests!B:B,A17,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E17">
+        <f>COUNTIFS(Tests!B:B,A17,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F17">
+        <f>COUNTIFS(Tests!B:B,A17,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B17" s="5">
-        <f>SUM(B2:B16)</f>
-        <v/>
-      </c>
-      <c r="C17" s="5">
-        <f>SUM(C2:C16)</f>
-        <v/>
-      </c>
-      <c r="D17" s="5">
-        <f>SUM(D2:D16)</f>
-        <v/>
-      </c>
-      <c r="E17" s="5">
-        <f>SUM(E2:E16)</f>
-        <v/>
-      </c>
-      <c r="F17" s="5">
-        <f>SUM(F2:F16)</f>
+      <c r="B18" s="5">
+        <f>SUM(B2:B17)</f>
+        <v/>
+      </c>
+      <c r="C18" s="5">
+        <f>SUM(C2:C17)</f>
+        <v/>
+      </c>
+      <c r="D18" s="5">
+        <f>SUM(D2:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="5">
+        <f>SUM(E2:E17)</f>
+        <v/>
+      </c>
+      <c r="F18" s="5">
+        <f>SUM(F2:F17)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
P5 step 8: remote support session through an outbound tunnel, owner only, time-limited (DL-235, 236)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/Chedam-Manual-Tests-P5.xlsx
+++ b/docs/testing/Chedam-Manual-Tests-P5.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$I$57</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2345,9 +2345,219 @@
       <c r="H51" s="3" t="inlineStr"/>
       <c r="I51" s="3" t="inlineStr"/>
     </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>S01</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (owner)</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>Home → Remote support → Add a key (paste a public key from the support PC: ssh-ed25519 …)</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Listed by name with the end of the key</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr"/>
+      <c r="H52" s="3" t="inlineStr"/>
+      <c r="I52" s="3" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>S02</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (owner)</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Let support in for 1 hour</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Support can sign in until …; an address …trycloudflare.com and a command to give support</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr"/>
+      <c r="H53" s="3" t="inlineStr"/>
+      <c r="I53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>S03</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Support PC (with cloudflared)</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Run the command shown</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>Signed in to the hub as chedam-support; sudo works; the owner's screen shows the sign-in</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr"/>
+      <c r="H54" s="3" t="inlineStr"/>
+      <c r="I54" s="3" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>S04</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (owner)</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>End now</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>The support PC's session is closed; signing in again fails</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr"/>
+      <c r="H55" s="3" t="inlineStr"/>
+      <c r="I55" s="3" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (owner)</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Let support in for 1 hour; wait past the end time</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>It ends by itself (Past sessions: ended by the end time); the key no longer works</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr"/>
+      <c r="H56" s="3" t="inlineStr"/>
+      <c r="I56" s="3" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Laptop (manager)</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Look for Remote support on Home</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>No tile (owner only)</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr"/>
+      <c r="H57" s="3" t="inlineStr"/>
+      <c r="I57" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I51"/>
-  <conditionalFormatting sqref="F2:F51">
+  <autoFilter ref="A1:I57"/>
+  <conditionalFormatting sqref="F2:F57">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -2362,7 +2572,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2376,7 +2586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2852,29 +3062,56 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="B18">
+        <f>COUNTIF(Tests!B:B,A18)</f>
+        <v/>
+      </c>
+      <c r="C18">
+        <f>COUNTIFS(Tests!B:B,A18,Tests!F:F,"Pass")</f>
+        <v/>
+      </c>
+      <c r="D18">
+        <f>COUNTIFS(Tests!B:B,A18,Tests!F:F,"Fail")</f>
+        <v/>
+      </c>
+      <c r="E18">
+        <f>COUNTIFS(Tests!B:B,A18,Tests!F:F,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="F18">
+        <f>COUNTIFS(Tests!B:B,A18,Tests!F:F,"Not tested")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B18" s="5">
-        <f>SUM(B2:B17)</f>
-        <v/>
-      </c>
-      <c r="C18" s="5">
-        <f>SUM(C2:C17)</f>
-        <v/>
-      </c>
-      <c r="D18" s="5">
-        <f>SUM(D2:D17)</f>
-        <v/>
-      </c>
-      <c r="E18" s="5">
-        <f>SUM(E2:E17)</f>
-        <v/>
-      </c>
-      <c r="F18" s="5">
-        <f>SUM(F2:F17)</f>
+      <c r="B19" s="5">
+        <f>SUM(B2:B18)</f>
+        <v/>
+      </c>
+      <c r="C19" s="5">
+        <f>SUM(C2:C18)</f>
+        <v/>
+      </c>
+      <c r="D19" s="5">
+        <f>SUM(D2:D18)</f>
+        <v/>
+      </c>
+      <c r="E19" s="5">
+        <f>SUM(E2:E18)</f>
+        <v/>
+      </c>
+      <c r="F19" s="5">
+        <f>SUM(F2:F18)</f>
         <v/>
       </c>
     </row>

</xml_diff>